<commit_message>
Improve monthly exports and add sourced AI electricity evidence
</commit_message>
<xml_diff>
--- a/dashboard/downloads/energy-demand.xlsx
+++ b/dashboard/downloads/energy-demand.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Informe" sheetId="1" r:id="R20d8acbffee64d3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos" sheetId="2" r:id="R23fa4e1453354681"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Informe" sheetId="1" r:id="Rcb06614313984979"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos" sheetId="2" r:id="Ra52e3124ba574960"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IA y energía" sheetId="3" r:id="R31be7bd125d64aa6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,7 +15,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="7">
+  <x:numFmts count="8">
     <x:numFmt numFmtId="200" formatCode="mmm yyyy"/>
     <x:numFmt numFmtId="201" formatCode="#,##0.0;[Red](#,##0.0);0.0"/>
     <x:numFmt numFmtId="202" formatCode="+0.0%;[Red]-0.0%;0.0%"/>
@@ -22,6 +23,7 @@
     <x:numFmt numFmtId="204" formatCode="+0.00;[Red]-0.00;0.00"/>
     <x:numFmt numFmtId="205" formatCode="0.000000"/>
     <x:numFmt numFmtId="206" formatCode="#,##0.000"/>
+    <x:numFmt numFmtId="207" formatCode="0"/>
   </x:numFmts>
   <x:fonts count="5">
     <x:font>
@@ -86,7 +88,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="31">
+  <x:cellXfs count="41">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -175,6 +177,36 @@
     </x:xf>
     <x:xf numFmtId="206" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="207" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -414,7 +446,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R797a13e6ec624553"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2b0a6867ba214f6e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1240,7 +1272,9 @@
       <x:c r="G41" s="2"/>
     </x:row>
     <x:row r="42" ht="23" customHeight="1">
-      <x:c r="A42" s="2"/>
+      <x:c r="A42" s="2" t="str">
+        <x:v>IA y electricidad: evidencia internacional y límites de atribución en la hoja IA y energía.</x:v>
+      </x:c>
       <x:c r="B42" s="2"/>
       <x:c r="C42" s="2"/>
       <x:c r="D42" s="2"/>
@@ -1255,7 +1289,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6e6fe321bc54cfd"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9ce5ea99a2f45ec"/>
 </x:worksheet>
 </file>
 
@@ -6316,7 +6350,593 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4cb09143a1d4a27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e8a12b6c7ea4c22"/>
   </x:tableParts>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFB86838"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="42" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="19" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="27" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="45" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="28" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="25" customHeight="1">
+      <x:c r="A1" s="32"/>
+      <x:c r="B1" s="32"/>
+      <x:c r="C1" s="32"/>
+      <x:c r="D1" s="32"/>
+      <x:c r="E1" s="32"/>
+      <x:c r="F1" s="32"/>
+      <x:c r="G1" s="32"/>
+    </x:row>
+    <x:row r="2" ht="35" customHeight="1">
+      <x:c r="A2" s="33" t="str">
+        <x:v>IA y electricidad: evidencia internacional y lectura argentina</x:v>
+      </x:c>
+      <x:c r="B2" s="32"/>
+      <x:c r="C2" s="32"/>
+      <x:c r="D2" s="32"/>
+      <x:c r="E2" s="32"/>
+      <x:c r="F2" s="32"/>
+      <x:c r="G2" s="32"/>
+    </x:row>
+    <x:row r="3" ht="32" customHeight="1">
+      <x:c r="A3" s="32" t="str">
+        <x:v>Revisión: 2026-09-24. El contexto internacional no representa la información disponible en cada mes histórico.</x:v>
+      </x:c>
+      <x:c r="B3" s="32"/>
+      <x:c r="C3" s="32"/>
+      <x:c r="D3" s="32"/>
+      <x:c r="E3" s="32"/>
+      <x:c r="F3" s="32"/>
+      <x:c r="G3" s="32"/>
+    </x:row>
+    <x:row r="4" ht="50" customHeight="1">
+      <x:c r="A4" s="32" t="str">
+        <x:v>Hay evidencia internacional de crecimiento eléctrico en centros de datos orientados a IA. Las series argentinas incorporadas no permiten medir qué parte del consumo sectorial corresponde a IA; no identificable no significa cero.</x:v>
+      </x:c>
+      <x:c r="B4" s="32"/>
+      <x:c r="C4" s="32"/>
+      <x:c r="D4" s="32"/>
+      <x:c r="E4" s="32"/>
+      <x:c r="F4" s="32"/>
+      <x:c r="G4" s="32"/>
+    </x:row>
+    <x:row r="5" ht="25" customHeight="1">
+      <x:c r="A5" s="32"/>
+      <x:c r="B5" s="32"/>
+      <x:c r="C5" s="32"/>
+      <x:c r="D5" s="32"/>
+      <x:c r="E5" s="32"/>
+      <x:c r="F5" s="32"/>
+      <x:c r="G5" s="32"/>
+    </x:row>
+    <x:row r="6" ht="25" customHeight="1">
+      <x:c r="A6" s="32" t="str">
+        <x:v>Mes local (vinculado a Informe)</x:v>
+      </x:c>
+      <x:c r="B6" s="34" t="n">
+        <x:f>'Informe'!B4</x:f>
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="C6" s="32"/>
+      <x:c r="D6" s="32"/>
+      <x:c r="E6" s="32"/>
+      <x:c r="F6" s="32"/>
+      <x:c r="G6" s="32"/>
+    </x:row>
+    <x:row r="7" ht="38" customHeight="1">
+      <x:c r="A7" s="8" t="str">
+        <x:v>Sector argentino</x:v>
+      </x:c>
+      <x:c r="B7" s="8" t="str">
+        <x:v>Interanual %</x:v>
+      </x:c>
+      <x:c r="C7" s="8" t="str">
+        <x:v>Atribución IA</x:v>
+      </x:c>
+      <x:c r="D7" s="32"/>
+      <x:c r="E7" s="32"/>
+      <x:c r="F7" s="32"/>
+      <x:c r="G7" s="32"/>
+    </x:row>
+    <x:row r="8" ht="25" customHeight="1">
+      <x:c r="A8" s="32" t="str">
+        <x:v>Comercio e industria</x:v>
+      </x:c>
+      <x:c r="B8" s="35" t="n">
+        <x:f>'Informe'!E11</x:f>
+        <x:v>-0.00524030458573745</x:v>
+      </x:c>
+      <x:c r="C8" s="32" t="str">
+        <x:v>No identificable</x:v>
+      </x:c>
+      <x:c r="D8" s="32" t="str">
+        <x:v>Variaciones sectoriales no son efectos de IA. No identificable no significa 0 GWh.</x:v>
+      </x:c>
+      <x:c r="E8" s="32"/>
+      <x:c r="F8" s="32"/>
+      <x:c r="G8" s="32"/>
+    </x:row>
+    <x:row r="9" ht="25" customHeight="1">
+      <x:c r="A9" s="32" t="str">
+        <x:v>Grandes usuarios</x:v>
+      </x:c>
+      <x:c r="B9" s="35" t="n">
+        <x:f>'Informe'!E12</x:f>
+        <x:v>0.12005734855625398</x:v>
+      </x:c>
+      <x:c r="C9" s="32" t="str">
+        <x:v>No identificable</x:v>
+      </x:c>
+      <x:c r="D9" s="32"/>
+      <x:c r="E9" s="32"/>
+      <x:c r="F9" s="32"/>
+      <x:c r="G9" s="32"/>
+    </x:row>
+    <x:row r="10" ht="25" customHeight="1">
+      <x:c r="A10" s="32"/>
+      <x:c r="B10" s="32"/>
+      <x:c r="C10" s="32"/>
+      <x:c r="D10" s="32"/>
+      <x:c r="E10" s="32"/>
+      <x:c r="F10" s="32"/>
+      <x:c r="G10" s="32"/>
+    </x:row>
+    <x:row r="11" ht="38" customHeight="1">
+      <x:c r="A11" s="8" t="str">
+        <x:v>Indicador</x:v>
+      </x:c>
+      <x:c r="B11" s="8" t="str">
+        <x:v>Ámbito / período</x:v>
+      </x:c>
+      <x:c r="C11" s="8" t="str">
+        <x:v>Valor</x:v>
+      </x:c>
+      <x:c r="D11" s="8" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="E11" s="8" t="str">
+        <x:v>Tipo de evidencia</x:v>
+      </x:c>
+      <x:c r="F11" s="8" t="str">
+        <x:v>Límite de interpretación</x:v>
+      </x:c>
+      <x:c r="G11" s="8" t="str">
+        <x:v>Fuente ID</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="80" customHeight="1">
+      <x:c r="A12" s="32" t="str">
+        <x:v>Electricidad de todos los centros de
+datos</x:v>
+      </x:c>
+      <x:c r="B12" s="32" t="str">
+        <x:v>Mundo
+2025</x:v>
+      </x:c>
+      <x:c r="C12" s="37" t="n">
+        <x:v>485</x:v>
+      </x:c>
+      <x:c r="D12" s="32" t="str">
+        <x:v>TWh</x:v>
+      </x:c>
+      <x:c r="E12" s="32" t="str">
+        <x:v>Estimación histórica</x:v>
+      </x:c>
+      <x:c r="F12" s="32" t="str">
+        <x:v>Incluye usos distintos de IA; no es una
+medición argentina.</x:v>
+      </x:c>
+      <x:c r="G12" s="32" t="str">
+        <x:v>IEA_AI_2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="80" customHeight="1">
+      <x:c r="A13" s="32" t="str">
+        <x:v>Crecimiento eléctrico de todos los
+centros de datos</x:v>
+      </x:c>
+      <x:c r="B13" s="32" t="str">
+        <x:v>Mundo
+2025 vs 2024</x:v>
+      </x:c>
+      <x:c r="C13" s="37" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D13" s="32" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="E13" s="32" t="str">
+        <x:v>Estimación histórica</x:v>
+      </x:c>
+      <x:c r="F13" s="32" t="str">
+        <x:v>No equivale al crecimiento atribuible
+exclusivamente a IA.</x:v>
+      </x:c>
+      <x:c r="G13" s="32" t="str">
+        <x:v>IEA_AI_2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="80" customHeight="1">
+      <x:c r="A14" s="32" t="str">
+        <x:v>Crecimiento eléctrico de centros de
+datos orientados a IA</x:v>
+      </x:c>
+      <x:c r="B14" s="32" t="str">
+        <x:v>Mundo
+2025 vs 2024</x:v>
+      </x:c>
+      <x:c r="C14" s="37" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="D14" s="32" t="str">
+        <x:v>%</x:v>
+      </x:c>
+      <x:c r="E14" s="32" t="str">
+        <x:v>Estimación histórica</x:v>
+      </x:c>
+      <x:c r="F14" s="32" t="str">
+        <x:v>Tasa de crecimiento, no participación de IA
+en los 485 TWh.</x:v>
+      </x:c>
+      <x:c r="G14" s="32" t="str">
+        <x:v>IEA_AI_2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="80" customHeight="1">
+      <x:c r="A15" s="32" t="str">
+        <x:v>Incremento eléctrico de todos los
+centros de datos</x:v>
+      </x:c>
+      <x:c r="B15" s="32" t="str">
+        <x:v>Mundo
+2025 vs 2024</x:v>
+      </x:c>
+      <x:c r="C15" s="37" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="D15" s="32" t="str">
+        <x:v>TWh</x:v>
+      </x:c>
+      <x:c r="E15" s="32" t="str">
+        <x:v>Estimación histórica
+aproximada</x:v>
+      </x:c>
+      <x:c r="F15" s="32" t="str">
+        <x:v>Todos los centros de datos; no solo IA.</x:v>
+      </x:c>
+      <x:c r="G15" s="32" t="str">
+        <x:v>IEA_GER_2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="80" customHeight="1">
+      <x:c r="A16" s="32" t="str">
+        <x:v>Incremento de la demanda eléctrica
+total</x:v>
+      </x:c>
+      <x:c r="B16" s="32" t="str">
+        <x:v>Mundo
+2025 vs 2024</x:v>
+      </x:c>
+      <x:c r="C16" s="37" t="n">
+        <x:v>800</x:v>
+      </x:c>
+      <x:c r="D16" s="32" t="str">
+        <x:v>TWh</x:v>
+      </x:c>
+      <x:c r="E16" s="32" t="str">
+        <x:v>Estimación histórica
+aproximada</x:v>
+      </x:c>
+      <x:c r="F16" s="32" t="str">
+        <x:v>Denominador mundial; no comparable
+directamente con un mes argentino.</x:v>
+      </x:c>
+      <x:c r="G16" s="32" t="str">
+        <x:v>IEA_GER_2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="80" customHeight="1">
+      <x:c r="A17" s="38" t="str">
+        <x:v>Electricidad de todos los centros de
+datos</x:v>
+      </x:c>
+      <x:c r="B17" s="38" t="str">
+        <x:v>Mundo
+2030</x:v>
+      </x:c>
+      <x:c r="C17" s="39" t="n">
+        <x:v>950</x:v>
+      </x:c>
+      <x:c r="D17" s="38" t="str">
+        <x:v>TWh</x:v>
+      </x:c>
+      <x:c r="E17" s="38" t="str">
+        <x:v>Proyección, no observado</x:v>
+      </x:c>
+      <x:c r="F17" s="38" t="str">
+        <x:v>Escenario de la AIE; no dato realizado ni
+pronóstico propio.</x:v>
+      </x:c>
+      <x:c r="G17" s="38" t="str">
+        <x:v>IEA_AI_2026</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="80" customHeight="1">
+      <x:c r="A18" s="32" t="str">
+        <x:v>Carta de intención OpenAI / Sur Energy
+para explorar un proyecto</x:v>
+      </x:c>
+      <x:c r="B18" s="32" t="str">
+        <x:v>Argentina
+2025-10-14</x:v>
+      </x:c>
+      <x:c r="C18" s="37"/>
+      <x:c r="D18" s="32" t="str">
+        <x:v>Sin GWh informados</x:v>
+      </x:c>
+      <x:c r="E18" s="32" t="str">
+        <x:v>Anuncio empresarial</x:v>
+      </x:c>
+      <x:c r="F18" s="32" t="str">
+        <x:v>Esta fuente acredita una intención; no
+aporta consumo medido ni acredita puesta en
+servicio.</x:v>
+      </x:c>
+      <x:c r="G18" s="32" t="str">
+        <x:v>OPENAI_AR_2025</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="25" customHeight="1">
+      <x:c r="A19" s="32"/>
+      <x:c r="B19" s="32"/>
+      <x:c r="C19" s="32"/>
+      <x:c r="D19" s="32"/>
+      <x:c r="E19" s="32"/>
+      <x:c r="F19" s="32"/>
+      <x:c r="G19" s="32"/>
+    </x:row>
+    <x:row r="20" ht="30" customHeight="1">
+      <x:c r="A20" s="32" t="str">
+        <x:v>Aporte aproximado de todos los centros de datos al aumento eléctrico mundial de 2025</x:v>
+      </x:c>
+      <x:c r="B20" s="32"/>
+      <x:c r="C20" s="32"/>
+      <x:c r="D20" s="32"/>
+      <x:c r="E20" s="32"/>
+      <x:c r="F20" s="32"/>
+      <x:c r="G20" s="32"/>
+    </x:row>
+    <x:row r="21" ht="25" customHeight="1">
+      <x:c r="A21" s="32" t="str">
+        <x:v>Incremento centros de datos (TWh)</x:v>
+      </x:c>
+      <x:c r="B21" s="32" t="n">
+        <x:f>C15</x:f>
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="C21" s="32"/>
+      <x:c r="D21" s="32" t="str">
+        <x:v>Cálculo propio con estimaciones redondeadas de AIE: 70 / 800. No mide el aporte exclusivo de IA ni la participación en el consumo total.</x:v>
+      </x:c>
+      <x:c r="E21" s="32"/>
+      <x:c r="F21" s="32"/>
+      <x:c r="G21" s="32"/>
+    </x:row>
+    <x:row r="22" ht="25" customHeight="1">
+      <x:c r="A22" s="32" t="str">
+        <x:v>Incremento mundial total (TWh)</x:v>
+      </x:c>
+      <x:c r="B22" s="32" t="n">
+        <x:f>C16</x:f>
+        <x:v>800</x:v>
+      </x:c>
+      <x:c r="C22" s="32"/>
+      <x:c r="D22" s="32"/>
+      <x:c r="E22" s="32"/>
+      <x:c r="F22" s="32"/>
+      <x:c r="G22" s="32"/>
+    </x:row>
+    <x:row r="23" ht="25" customHeight="1">
+      <x:c r="A23" s="32" t="str">
+        <x:v>Aporte al incremento mundial (%)</x:v>
+      </x:c>
+      <x:c r="B23" s="40" t="n">
+        <x:f>B21/B22</x:f>
+        <x:v>0.0875</x:v>
+      </x:c>
+      <x:c r="C23" s="32"/>
+      <x:c r="D23" s="32"/>
+      <x:c r="E23" s="32"/>
+      <x:c r="F23" s="32"/>
+      <x:c r="G23" s="32"/>
+    </x:row>
+    <x:row r="24" ht="25" customHeight="1">
+      <x:c r="A24" s="32"/>
+      <x:c r="B24" s="32"/>
+      <x:c r="C24" s="32"/>
+      <x:c r="D24" s="32"/>
+      <x:c r="E24" s="32"/>
+      <x:c r="F24" s="32"/>
+      <x:c r="G24" s="32"/>
+    </x:row>
+    <x:row r="25" ht="65" customHeight="1">
+      <x:c r="A25" s="32" t="str">
+        <x:v>Centros de datos no equivale a industria ni todo centro de datos se dedica a IA. El cómputo contratado por una empresa argentina puede ejecutarse fuera del país. Adoptar IA tampoco implica necesariamente mayor consumo neto de la fábrica: deben medirse tanto el cómputo como los cambios de eficiencia y producción.</x:v>
+      </x:c>
+      <x:c r="B25" s="32"/>
+      <x:c r="C25" s="32"/>
+      <x:c r="D25" s="32"/>
+      <x:c r="E25" s="32"/>
+      <x:c r="F25" s="32"/>
+      <x:c r="G25" s="32"/>
+    </x:row>
+    <x:row r="26" ht="70" customHeight="1">
+      <x:c r="A26" s="32" t="str">
+        <x:v>Para estimar una relación local hacen falta consumos mensuales por establecimiento, ubicación del cómputo, fecha de adopción de IA y proporción de carga dedicada a IA. Comparar establecimientos semejantes antes y después, controlando producción, clima, calendario y tarifas; verificar tendencias previas antes de interpretar causalmente.</x:v>
+      </x:c>
+      <x:c r="B26" s="32"/>
+      <x:c r="C26" s="32"/>
+      <x:c r="D26" s="32"/>
+      <x:c r="E26" s="32"/>
+      <x:c r="F26" s="32"/>
+      <x:c r="G26" s="32"/>
+    </x:row>
+    <x:row r="27" ht="25" customHeight="1">
+      <x:c r="A27" s="32"/>
+      <x:c r="B27" s="32"/>
+      <x:c r="C27" s="32"/>
+      <x:c r="D27" s="32"/>
+      <x:c r="E27" s="32"/>
+      <x:c r="F27" s="32"/>
+      <x:c r="G27" s="32"/>
+    </x:row>
+    <x:row r="28" ht="30" customHeight="1">
+      <x:c r="A28" s="32" t="str">
+        <x:v>Fuentes de los indicadores (la fecha de revisión no es la del dato)</x:v>
+      </x:c>
+      <x:c r="B28" s="32"/>
+      <x:c r="C28" s="32"/>
+      <x:c r="D28" s="32"/>
+      <x:c r="E28" s="32"/>
+      <x:c r="F28" s="32"/>
+      <x:c r="G28" s="32"/>
+    </x:row>
+    <x:row r="29" ht="30" customHeight="1">
+      <x:c r="A29" s="32" t="str">
+        <x:v>IEA_AI_2026: AIE / IEA. Key Questions on Energy and AI (2026)</x:v>
+      </x:c>
+      <x:c r="B29" s="32"/>
+      <x:c r="C29" s="32"/>
+      <x:c r="D29" s="32"/>
+      <x:c r="E29" s="32"/>
+      <x:c r="F29" s="32"/>
+      <x:c r="G29" s="32"/>
+    </x:row>
+    <x:row r="30" ht="35" customHeight="1">
+      <x:c r="A30" s="32" t="str">
+        <x:v>https://www.iea.org/reports/key-questions-on-energy-and-ai/executive-summary</x:v>
+      </x:c>
+      <x:c r="B30" s="32"/>
+      <x:c r="C30" s="32"/>
+      <x:c r="D30" s="32"/>
+      <x:c r="E30" s="32"/>
+      <x:c r="F30" s="32"/>
+      <x:c r="G30" s="32"/>
+    </x:row>
+    <x:row r="31" ht="30" customHeight="1">
+      <x:c r="A31" s="32" t="str">
+        <x:v>IEA_GER_2026: AIE / IEA. Global Energy Review 2026 — Electricity demand</x:v>
+      </x:c>
+      <x:c r="B31" s="32"/>
+      <x:c r="C31" s="32"/>
+      <x:c r="D31" s="32"/>
+      <x:c r="E31" s="32"/>
+      <x:c r="F31" s="32"/>
+      <x:c r="G31" s="32"/>
+    </x:row>
+    <x:row r="32" ht="35" customHeight="1">
+      <x:c r="A32" s="32" t="str">
+        <x:v>https://www.iea.org/reports/global-energy-review-2026/electricity-demand</x:v>
+      </x:c>
+      <x:c r="B32" s="32"/>
+      <x:c r="C32" s="32"/>
+      <x:c r="D32" s="32"/>
+      <x:c r="E32" s="32"/>
+      <x:c r="F32" s="32"/>
+      <x:c r="G32" s="32"/>
+    </x:row>
+    <x:row r="33" ht="30" customHeight="1">
+      <x:c r="A33" s="32" t="str">
+        <x:v>OPENAI_AR_2025: OpenAI. Argentina’s AI opportunity — 14 octubre 2025</x:v>
+      </x:c>
+      <x:c r="B33" s="32"/>
+      <x:c r="C33" s="32"/>
+      <x:c r="D33" s="32"/>
+      <x:c r="E33" s="32"/>
+      <x:c r="F33" s="32"/>
+      <x:c r="G33" s="32"/>
+    </x:row>
+    <x:row r="34" ht="35" customHeight="1">
+      <x:c r="A34" s="32" t="str">
+        <x:v>https://openai.com/global-affairs/argentinas-ai-opportunity/</x:v>
+      </x:c>
+      <x:c r="B34" s="32"/>
+      <x:c r="C34" s="32"/>
+      <x:c r="D34" s="32"/>
+      <x:c r="E34" s="32"/>
+      <x:c r="F34" s="32"/>
+      <x:c r="G34" s="32"/>
+    </x:row>
+    <x:row r="35" ht="25" customHeight="1">
+      <x:c r="A35" s="32"/>
+      <x:c r="B35" s="32"/>
+      <x:c r="C35" s="32"/>
+      <x:c r="D35" s="32"/>
+      <x:c r="E35" s="32"/>
+      <x:c r="F35" s="32"/>
+      <x:c r="G35" s="32"/>
+    </x:row>
+    <x:row r="36" ht="32" customHeight="1">
+      <x:c r="A36" s="32" t="str">
+        <x:v>Unidades: 1 TWh = 1.000 GWh. La tabla combina ámbitos y períodos distintos: sus filas no se suman.</x:v>
+      </x:c>
+      <x:c r="B36" s="32"/>
+      <x:c r="C36" s="32"/>
+      <x:c r="D36" s="32"/>
+      <x:c r="E36" s="32"/>
+      <x:c r="F36" s="32"/>
+      <x:c r="G36" s="32"/>
+    </x:row>
+    <x:row r="37" ht="25" customHeight="1">
+      <x:c r="A37" s="32"/>
+      <x:c r="B37" s="32"/>
+      <x:c r="C37" s="32"/>
+      <x:c r="D37" s="32"/>
+      <x:c r="E37" s="32"/>
+      <x:c r="F37" s="32"/>
+      <x:c r="G37" s="32"/>
+    </x:row>
+    <x:row r="38" ht="25" customHeight="1">
+      <x:c r="A38" s="32"/>
+      <x:c r="B38" s="32"/>
+      <x:c r="C38" s="32"/>
+      <x:c r="D38" s="32"/>
+      <x:c r="E38" s="32"/>
+      <x:c r="F38" s="32"/>
+      <x:c r="G38" s="32"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A2:G2"/>
+    <x:mergeCell ref="A3:G3"/>
+    <x:mergeCell ref="A4:G4"/>
+    <x:mergeCell ref="D8:G9"/>
+    <x:mergeCell ref="A20:G20"/>
+    <x:mergeCell ref="D21:G23"/>
+    <x:mergeCell ref="A25:G25"/>
+    <x:mergeCell ref="A26:G26"/>
+    <x:mergeCell ref="A28:G28"/>
+    <x:mergeCell ref="A29:G29"/>
+    <x:mergeCell ref="A30:G30"/>
+    <x:mergeCell ref="A31:G31"/>
+    <x:mergeCell ref="A32:G32"/>
+    <x:mergeCell ref="A33:G33"/>
+    <x:mergeCell ref="A34:G34"/>
+    <x:mergeCell ref="A36:G36"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>